<commit_message>
add customer successful from excel
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/Testcase.xlsx
+++ b/src/test/resources/excel/Testcase.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/Desktop/learn/DataDrivenFramework/src/test/resources/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4D7E2AE9-541B-4A4D-9FD3-16FBD2EA3132}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C826F5-81A1-734F-B685-3571CBAA790D}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15800" xr2:uid="{6053CA53-42B5-BB40-92FC-8EE2CDB42BB3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="addCustomer" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -22,6 +22,32 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>Kieu</t>
+  </si>
+  <si>
+    <t>Trang</t>
+  </si>
+  <si>
+    <t>alert</t>
+  </si>
+  <si>
+    <t>Customer added successfully</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -371,9 +397,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{901EBAC3-1131-0C4B-AF4B-6772091AA3E4}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>3112</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>